<commit_message>
changed distance from the center to 30º
</commit_message>
<xml_diff>
--- a/Components_parameters.xlsx
+++ b/Components_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\H-IBL.TaskPretest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78903065-E6A8-48F3-AB23-FF76D653354B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB57F29-4A72-4F42-96ED-4F2B41DF0083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -97,18 +97,12 @@
     <t>gauss</t>
   </si>
   <si>
-    <t>(15, 0)</t>
-  </si>
-  <si>
     <t>0.16</t>
   </si>
   <si>
     <t>0.32</t>
   </si>
   <si>
-    <t>(-15,0)</t>
-  </si>
-  <si>
     <t>0.01</t>
   </si>
   <si>
@@ -116,6 +110,12 @@
   </si>
   <si>
     <t>0.04</t>
+  </si>
+  <si>
+    <t>(30, 0)</t>
+  </si>
+  <si>
+    <t>(-30,0)</t>
   </si>
 </sst>
 </file>
@@ -482,7 +482,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -517,7 +517,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -552,10 +552,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -587,10 +587,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
@@ -622,10 +622,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -657,10 +657,10 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
@@ -692,10 +692,10 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
@@ -727,10 +727,10 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
@@ -762,7 +762,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
@@ -797,7 +797,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
         <v>8</v>
@@ -832,10 +832,10 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
         <v>17</v>
-      </c>
-      <c r="B12" t="s">
-        <v>18</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
@@ -867,10 +867,10 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
@@ -902,10 +902,10 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
@@ -937,10 +937,10 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
         <v>11</v>
@@ -972,7 +972,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B16">
         <v>1</v>
@@ -1007,7 +1007,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B17">
         <v>1</v>

</xml_diff>